<commit_message>
feat: formato oficial de tablas (bordes completos, semestre AAAA-S y fuente Zurich Cn BT 11)
- Bordes en todas las celdas de Sistematizacion y Certificados (Modo 3 y Modo 5).
- La celda de fin de clase conserva los 3 lados finos + borde inferior grueso.
- Columna Semestre en formato oficial AAAA-S (ej. 2026-1) en Certificados.
- Nueva regla de semestre: S1 = 1 nov-30 abr; S2 = 1 may-31 oct.
- Fuente oficial de Certificados: Zurich Cn BT 11.
- Fix: parseo de fechas ISO (AAAA-MM-DD) que devolvia None.
- Tests actualizados (34/34 OK) y AGENTS.md agregado.
</commit_message>
<xml_diff>
--- a/tests/fixtures/synthetic_certificados.xlsx
+++ b/tests/fixtures/synthetic_certificados.xlsx
@@ -530,8 +530,10 @@
       <c r="J2" t="n">
         <v>2026</v>
       </c>
-      <c r="K2" t="n">
-        <v>1</v>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-1</t>
+        </is>
       </c>
       <c r="L2" t="n">
         <v>1</v>

</xml_diff>